<commit_message>
Updated on 12-11-2023 at 21:23
</commit_message>
<xml_diff>
--- a/data/cubic_latex.xlsx
+++ b/data/cubic_latex.xlsx
@@ -565,7 +565,7 @@
         <v>0.898</v>
       </c>
       <c r="C13" t="n">
-        <v>-6.385</v>
+        <v>6.791</v>
       </c>
     </row>
     <row r="14">
@@ -653,7 +653,7 @@
         <v>1.551</v>
       </c>
       <c r="C21" t="n">
-        <v>-8.02</v>
+        <v>6.15</v>
       </c>
     </row>
     <row r="22">
@@ -950,7 +950,7 @@
         <v>3.755</v>
       </c>
       <c r="C48" t="n">
-        <v>8.228999999999999</v>
+        <v>22.576</v>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
Updated on 12-11-2023 at 21:35
</commit_message>
<xml_diff>
--- a/data/cubic_latex.xlsx
+++ b/data/cubic_latex.xlsx
@@ -466,7 +466,7 @@
         <v>0.163</v>
       </c>
       <c r="C4" t="n">
-        <v>6.136</v>
+        <v>1.078</v>
       </c>
     </row>
     <row r="5">
@@ -554,7 +554,7 @@
         <v>0.8159999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>0.364</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -565,7 +565,7 @@
         <v>0.898</v>
       </c>
       <c r="C13" t="n">
-        <v>6.791</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -576,7 +576,7 @@
         <v>0.98</v>
       </c>
       <c r="C14" t="n">
-        <v>0.044</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -587,7 +587,7 @@
         <v>1.061</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -598,7 +598,7 @@
         <v>1.143</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.29</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -609,7 +609,7 @@
         <v>1.224</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.434</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
@@ -620,7 +620,7 @@
         <v>1.306</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.585</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19">
@@ -631,7 +631,7 @@
         <v>1.388</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.719</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
@@ -642,7 +642,7 @@
         <v>1.469</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.826</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -653,7 +653,7 @@
         <v>1.551</v>
       </c>
       <c r="C21" t="n">
-        <v>6.15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -840,7 +840,7 @@
         <v>2.939</v>
       </c>
       <c r="C38" t="n">
-        <v>-6.461</v>
+        <v>3.401</v>
       </c>
     </row>
     <row r="39">
@@ -950,7 +950,7 @@
         <v>3.755</v>
       </c>
       <c r="C48" t="n">
-        <v>22.576</v>
+        <v>15.395</v>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
Updated on 12-12-2023 at 12:18
</commit_message>
<xml_diff>
--- a/data/cubic_latex.xlsx
+++ b/data/cubic_latex.xlsx
@@ -466,7 +466,7 @@
         <v>0.163</v>
       </c>
       <c r="C4" t="n">
-        <v>1.078</v>
+        <v>6.136</v>
       </c>
     </row>
     <row r="5">
@@ -554,7 +554,7 @@
         <v>0.8159999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>10</v>
+        <v>0.364</v>
       </c>
     </row>
     <row r="13">
@@ -565,7 +565,7 @@
         <v>0.898</v>
       </c>
       <c r="C13" t="n">
-        <v>10</v>
+        <v>-6.385</v>
       </c>
     </row>
     <row r="14">
@@ -576,7 +576,7 @@
         <v>0.98</v>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>0.044</v>
       </c>
     </row>
     <row r="15">
@@ -587,7 +587,7 @@
         <v>1.061</v>
       </c>
       <c r="C15" t="n">
-        <v>10</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="16">
@@ -598,7 +598,7 @@
         <v>1.143</v>
       </c>
       <c r="C16" t="n">
-        <v>10</v>
+        <v>-0.29</v>
       </c>
     </row>
     <row r="17">
@@ -609,7 +609,7 @@
         <v>1.224</v>
       </c>
       <c r="C17" t="n">
-        <v>10</v>
+        <v>-0.434</v>
       </c>
     </row>
     <row r="18">
@@ -620,7 +620,7 @@
         <v>1.306</v>
       </c>
       <c r="C18" t="n">
-        <v>10</v>
+        <v>-0.585</v>
       </c>
     </row>
     <row r="19">
@@ -631,7 +631,7 @@
         <v>1.388</v>
       </c>
       <c r="C19" t="n">
-        <v>10</v>
+        <v>-0.719</v>
       </c>
     </row>
     <row r="20">
@@ -642,7 +642,7 @@
         <v>1.469</v>
       </c>
       <c r="C20" t="n">
-        <v>10</v>
+        <v>-0.826</v>
       </c>
     </row>
     <row r="21">
@@ -653,7 +653,7 @@
         <v>1.551</v>
       </c>
       <c r="C21" t="n">
-        <v>10</v>
+        <v>-8.02</v>
       </c>
     </row>
     <row r="22">
@@ -840,7 +840,7 @@
         <v>2.939</v>
       </c>
       <c r="C38" t="n">
-        <v>3.401</v>
+        <v>-6.461</v>
       </c>
     </row>
     <row r="39">
@@ -950,7 +950,7 @@
         <v>3.755</v>
       </c>
       <c r="C48" t="n">
-        <v>15.395</v>
+        <v>8.228999999999999</v>
       </c>
     </row>
     <row r="49">

</xml_diff>